<commit_message>
Publish ready daily articles 2026-09-14
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -452,7 +452,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6">
@@ -482,7 +482,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>153</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>153</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10">
@@ -536,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -610,6 +610,11 @@
           <t>planning_reasoning</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>source_list</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -617,22 +622,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>The SaaS Apocalypse Is Real. Causal AI Is the Escape Route</t>
+          <t>open-code-review Review 2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>The SaaS Apocalypse Is Real. Causal AI Is the Escape Route</t>
+          <t>open-code-review Review 2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>the-saas-apocalypse-is-real-causal-ai-is-the-escape-route</t>
+          <t>open-code-review-review-2026</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>mixed informational and commercial</t>
+          <t>commercial research</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -642,11 +647,11 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The SaaS Apocalypse Is Real. Causal AI Is the Escape Route</t>
+          <t>open-code-review Review 2026</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>54.1</v>
+        <v>64.8</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -658,7 +663,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -668,12 +673,17 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>["the saas apocalypse is real causal ai is the escape route comparison", "the saas apocalypse is real causal ai is the escape route faq", "how to use the saas apocalypse is real causal ai is the escape route", "the saas apocalypse is real causal ai is the escape route alternatives", "the saas apocalypse is real causal ai is the escape route pricing"]</t>
+          <t>["open-code-review review 2026 alternatives", "how to use open-code-review review 2026", "open-code-review review 2026 faq", "open-code-review review 2026 comparison", "open-code-review review 2026 pricing"]</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>["Detected search intent 'commercial' from the query.", "Intent confidence 0.0; article-type confidence 0.0.", "Detected search intent 'informational' from the query.", "Intent depth classified as shallow based on query specificity.", "Scope classified as broad based on narrowing terms and product intent.", "Buyer journey stage is awareness and funnel stage is top."]</t>
+          <t>["Detected search intent 'commercial' from the query.", "Matched intent terms: review.", "Matched article-type terms: review.", "Intent confidence 0.9; article-type confidence 0.95.", "Detected search intent 'commercial' from the query.", "Intent depth classified as shallow based on query specificity."]</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>["github_trending"]</t>
         </is>
       </c>
     </row>
@@ -683,17 +693,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>best ai productivity software</t>
+          <t>TradingAgents Review 2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>best ai productivity software</t>
+          <t>TradingAgents Review 2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>best-ai-productivity-software</t>
+          <t>tradingagents-review-2026</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -703,16 +713,16 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>AI Software</t>
+          <t>AI Agents</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>best ai productivity software</t>
+          <t>TradingAgents Review 2026</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>51.7</v>
+        <v>58.5</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -724,22 +734,27 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>listicle</t>
+          <t>review</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>["how to use best ai productivity software", "best ai productivity software comparison", "best ai productivity software faq", "best ai productivity software alternatives", "best ai productivity software pricing"]</t>
+          <t>["tradingagents review 2026 pricing", "tradingagents review 2026 alternatives", "how to use tradingagents review 2026", "tradingagents review 2026 comparison", "tradingagents review 2026 faq"]</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>["Detected search intent 'commercial' from the query.", "Matched intent terms: best.", "Matched article-type terms: best.", "Intent confidence 0.95; article-type confidence 1.25.", "Detected search intent 'commercial' from the query.", "Intent depth classified as medium based on query specificity."]</t>
+          <t>["Detected search intent 'commercial' from the query.", "Matched intent terms: review.", "Matched article-type terms: review.", "Intent confidence 0.9; article-type confidence 0.95.", "Detected search intent 'commercial' from the query.", "Intent depth classified as shallow based on query specificity."]</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>["github_trending"]</t>
         </is>
       </c>
     </row>
@@ -749,22 +764,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>best ai meeting software</t>
+          <t>Import AI 465: Open vs closed gaps; Kimi K3; Demis' big policy plan</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>best ai meeting software</t>
+          <t>Import AI 465: Open vs closed gaps; Kimi K3; Demis' big policy plan</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>best-ai-meeting-software</t>
+          <t>import-ai-465-open-vs-closed-gaps-kimi-k3-demis-big-policy-plan</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>commercial research</t>
+          <t>comparison</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -774,15 +789,15 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>best ai meeting software</t>
+          <t>Import AI 465: Open vs closed gaps; Kimi K3; Demis' big policy plan</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>50.5</v>
+        <v>53.3</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="J4" t="n">
@@ -795,17 +810,22 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>listicle</t>
+          <t>comparison</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>["best ai meeting software alternatives", "best ai meeting software comparison", "best ai meeting software pricing", "how to use best ai meeting software", "best ai meeting software faq"]</t>
+          <t>["how to use import ai 465 open vs closed gaps kimi k3 demis big policy plan", "import ai 465 open vs closed gaps kimi k3 demis big policy plan faq", "import ai 465 open vs closed gaps kimi k3 demis big policy plan comparison", "import ai 465 open vs closed gaps kimi k3 demis big policy plan pricing", "import ai 465 open vs closed gaps kimi k3 demis big policy plan alternatives"]</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>["Detected search intent 'commercial' from the query.", "Matched intent terms: best.", "Matched article-type terms: best.", "Intent confidence 0.95; article-type confidence 1.25.", "Detected search intent 'commercial' from the query.", "Intent depth classified as medium based on query specificity."]</t>
+          <t>["Detected search intent 'commercial' from the query.", "Matched intent terms: vs.", "Matched article-type terms: vs.", "Intent confidence 0.95; article-type confidence 1.28.", "Detected search intent 'commercial' from the query.", "Intent depth classified as medium based on query specificity."]</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>["ai_newsletters"]</t>
         </is>
       </c>
     </row>
@@ -815,22 +835,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>best ai voice software</t>
+          <t>When AI Does the Work: How SaaS Business Models Have to Change</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>best ai voice software</t>
+          <t>When AI Does the Work: How SaaS Business Models Have to Change</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>best-ai-voice-software</t>
+          <t>when-ai-does-the-work-how-saas-business-models-have-to-change</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>commercial research</t>
+          <t>mixed informational and commercial</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -840,11 +860,11 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>best ai voice software</t>
+          <t>When AI Does the Work: How SaaS Business Models Have to Change</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>50.5</v>
+        <v>52.9</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -861,17 +881,22 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>listicle</t>
+          <t>review</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>["best ai voice software pricing", "best ai voice software alternatives", "best ai voice software faq", "how to use best ai voice software", "best ai voice software comparison"]</t>
+          <t>["how to use when ai does the work how saas business models have to change", "when ai does the work how saas business models have to change pricing", "when ai does the work how saas business models have to change alternatives", "when ai does the work how saas business models have to change comparison", "when ai does the work how saas business models have to change faq"]</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>["Detected search intent 'commercial' from the query.", "Matched intent terms: best.", "Matched article-type terms: best.", "Intent confidence 0.95; article-type confidence 1.25.", "Detected search intent 'commercial' from the query.", "Intent depth classified as medium based on query specificity."]</t>
+          <t>["Detected search intent 'commercial' from the query.", "Intent confidence 0.0; article-type confidence 0.0.", "Detected search intent 'informational' from the query.", "Intent depth classified as shallow based on query specificity.", "Scope classified as broad based on narrowing terms and product intent.", "Buyer journey stage is awareness and funnel stage is top."]</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>["bing_trending"]</t>
         </is>
       </c>
     </row>
@@ -881,17 +906,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Impartner Redefines Partner Marketing Automation with Full Automation, AdTech and AI to Drive Measurable Revenue</t>
+          <t>Paid: Reshaping SaaS Monetisation for Agentic AI Models</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Impartner Redefines Partner Marketing Automation with Full Automation, AdTech and AI to Drive Measurable Revenue</t>
+          <t>Paid: Reshaping SaaS Monetisation for Agentic AI Models</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>impartner-redefines-partner-marketing-automation-with-full-automation-adtech-and-ai-to-drive-measurable-revenue</t>
+          <t>paid-reshaping-saas-monetisation-for-agentic-ai-models</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -901,16 +926,16 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>AI Software</t>
+          <t>AI Agents</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Impartner Redefines Partner Marketing Automation with Full Automation, AdTech and AI to Drive Measurable Revenue</t>
+          <t>Paid: Reshaping SaaS Monetisation for Agentic AI Models</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>50.3</v>
+        <v>52.5</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -932,12 +957,17 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>["how to use impartner redefines partner marketing automation with full automation adtech and ai to drive measurable revenue", "impartner redefines partner marketing automation with full automation adtech and ai to drive measurable revenue faq", "impartner redefines partner marketing automation with full automation adtech and ai to drive measurable revenue alternatives", "impartner redefines partner marketing automation with full automation adtech and ai to drive measurable revenue comparison", "impartner redefines partner marketing automation with full automation adtech and ai to drive measurable revenue pricing"]</t>
+          <t>["paid reshaping saas monetisation for agentic ai models pricing", "paid reshaping saas monetisation for agentic ai models comparison", "paid reshaping saas monetisation for agentic ai models alternatives", "how to use paid reshaping saas monetisation for agentic ai models", "paid reshaping saas monetisation for agentic ai models faq"]</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
           <t>["Detected search intent 'commercial' from the query.", "Intent confidence 0.0; article-type confidence 0.0.", "Detected search intent 'informational' from the query.", "Intent depth classified as shallow based on query specificity.", "Scope classified as broad based on narrowing terms and product intent.", "Buyer journey stage is awareness and funnel stage is top."]</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>["bing_trending"]</t>
         </is>
       </c>
     </row>
@@ -947,36 +977,36 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AI coding tokens could soon cost as much as salaries</t>
+          <t>5 AI Tools That Are Secretly Replacing Your Job Right Now</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AI coding tokens could soon cost as much as salaries</t>
+          <t>5 AI Tools That Are Secretly Replacing Your Job Right Now</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ai-coding-tokens-could-soon-cost-as-much-as-salaries</t>
+          <t>5-ai-tools-that-are-secretly-replacing-your-job-right-now</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>commercial investigation</t>
+          <t>commercial research</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>AI Coding</t>
+          <t>AI Software</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>AI coding tokens could soon cost as much as salaries</t>
+          <t>5 AI Tools That Are Secretly Replacing Your Job Right Now</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>49.8</v>
+        <v>52.1</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -993,17 +1023,22 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>listicle</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>["ai coding tokens could soon cost as much as salaries pricing", "ai coding tokens could soon cost as much as salaries faq", "how to use ai coding tokens could soon cost as much as salaries", "ai coding tokens could soon cost as much as salaries comparison", "ai coding tokens could soon cost as much as salaries alternatives"]</t>
+          <t>["how to use 5 ai tools that are secretly replacing your job right now", "5 ai tools that are secretly replacing your job right now faq", "5 ai tools that are secretly replacing your job right now comparison", "5 ai tools that are secretly replacing your job right now pricing", "5 ai tools that are secretly replacing your job right now alternatives"]</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>["Detected search intent 'transactional' from the query.", "Matched intent terms: cost.", "Matched article-type terms: cost.", "Intent confidence 0.95; article-type confidence 0.95.", "Detected search intent 'transactional' from the query.", "Intent depth classified as deep based on query specificity."]</t>
+          <t>["Detected search intent 'commercial' from the query.", "Intent confidence 0.0; article-type confidence 0.0.", "Detected search intent 'informational' from the query.", "Intent depth classified as shallow based on query specificity.", "Scope classified as broad based on narrowing terms and product intent.", "Buyer journey stage is awareness and funnel stage is top."]</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>["bing_trending"]</t>
         </is>
       </c>
     </row>
@@ -1013,22 +1048,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>How AI is upending SaaS tools</t>
+          <t>Adobe Acquires Indian AI Startup Rilo for Marketing Automation</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>How AI is upending SaaS tools</t>
+          <t>Adobe Acquires Indian AI Startup Rilo for Marketing Automation</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>how-ai-is-upending-saas-tools</t>
+          <t>adobe-acquires-indian-ai-startup-rilo-for-marketing-automation</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>commercial research</t>
+          <t>mixed informational and commercial</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1038,11 +1073,11 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>How AI is upending SaaS tools</t>
+          <t>Adobe Acquires Indian AI Startup Rilo for Marketing Automation</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>49.3</v>
+        <v>50.1</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -1059,17 +1094,22 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>listicle</t>
+          <t>news/update</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>["how ai is upending saas tools pricing", "how ai is upending saas tools faq", "how ai is upending saas tools alternatives", "how to use how ai is upending saas tools", "how ai is upending saas tools comparison"]</t>
+          <t>["adobe acquires indian ai startup rilo for marketing automation alternatives", "adobe acquires indian ai startup rilo for marketing automation faq", "adobe acquires indian ai startup rilo for marketing automation pricing", "adobe acquires indian ai startup rilo for marketing automation comparison", "how to use adobe acquires indian ai startup rilo for marketing automation"]</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
           <t>["Detected search intent 'commercial' from the query.", "Intent confidence 0.0; article-type confidence 0.0.", "Detected search intent 'informational' from the query.", "Intent depth classified as shallow based on query specificity.", "Scope classified as broad based on narrowing terms and product intent.", "Buyer journey stage is awareness and funnel stage is top."]</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>["bing_trending"]</t>
         </is>
       </c>
     </row>
@@ -1079,17 +1119,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Shopify launches AI-powered marketing automation tool</t>
+          <t>Organizations build software in-house using agentic coding tools instead of buying</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Shopify launches AI-powered marketing automation tool</t>
+          <t>Organizations build software in-house using agentic coding tools instead of buying</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>shopify-launches-ai-powered-marketing-automation-tool</t>
+          <t>organizations-build-software-in-house-using-agentic-coding-tools-instead-of-buying</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1099,16 +1139,16 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>AI Software</t>
+          <t>AI Coding</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Shopify launches AI-powered marketing automation tool</t>
+          <t>Organizations build software in-house using agentic coding tools instead of buying</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>48.9</v>
+        <v>49.7</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1125,17 +1165,22 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>news/update</t>
+          <t>listicle</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>["shopify launches ai-powered marketing automation tool comparison", "how to use shopify launches ai-powered marketing automation tool", "shopify launches ai-powered marketing automation tool alternatives", "shopify launches ai-powered marketing automation tool faq", "shopify launches ai-powered marketing automation tool pricing"]</t>
+          <t>["organizations build software in-house using agentic coding tools instead of buying comparison", "how to use organizations build software in-house using agentic coding tools instead of buying", "organizations build software in-house using agentic coding tools instead of buying alternatives", "organizations build software in-house using agentic coding tools instead of buying pricing", "organizations build software in-house using agentic coding tools instead of buying faq"]</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>["Detected search intent 'commercial' from the query.", "Intent confidence 0.0; article-type confidence 0.0.", "Detected search intent 'informational' from the query.", "Intent depth classified as shallow based on query specificity.", "Scope classified as broad based on narrowing terms and product intent.", "Buyer journey stage is awareness and funnel stage is top."]</t>
+          <t>["Detected search intent 'transactional' from the query.", "Matched intent terms: buy.", "Intent confidence 0.9; article-type confidence 0.0.", "Detected search intent 'transactional' from the query.", "Intent depth classified as deep based on query specificity.", "Scope classified as narrow based on narrowing terms and product intent."]</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>["bing_trending"]</t>
         </is>
       </c>
     </row>
@@ -1145,17 +1190,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>best ai meeting tools</t>
+          <t>We Tested the 10 Best AI Productivity Tools in 2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>best ai meeting tools</t>
+          <t>We Tested the 10 Best AI Productivity Tools in 2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>best-ai-meeting-tools</t>
+          <t>we-tested-the-10-best-ai-productivity-tools-in-2026</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1170,11 +1215,11 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>best ai meeting tools</t>
+          <t>We Tested the 10 Best AI Productivity Tools in 2026</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>48.8</v>
+        <v>49.7</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1196,12 +1241,17 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>["how to use best ai meeting tools", "best ai meeting tools comparison", "best ai meeting tools alternatives", "best ai meeting tools faq", "best ai meeting tools pricing"]</t>
+          <t>["we tested the 10 best ai productivity tools in 2026 comparison", "we tested the 10 best ai productivity tools in 2026 pricing", "we tested the 10 best ai productivity tools in 2026 alternatives", "how to use we tested the 10 best ai productivity tools in 2026", "we tested the 10 best ai productivity tools in 2026 faq"]</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
           <t>["Detected search intent 'commercial' from the query.", "Matched intent terms: best.", "Matched article-type terms: best.", "Intent confidence 0.95; article-type confidence 1.25.", "Detected search intent 'commercial' from the query.", "Intent depth classified as medium based on query specificity."]</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>["bing_trending"]</t>
         </is>
       </c>
     </row>
@@ -1211,36 +1261,36 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>AI coding costs could exceed developer salaries by 2028</t>
+          <t>Zoho adds AI tools to Catalyst cloud platform</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AI coding costs could exceed developer salaries by 2028</t>
+          <t>Zoho adds AI tools to Catalyst cloud platform</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ai-coding-costs-could-exceed-developer-salaries-by-2028</t>
+          <t>zoho-adds-ai-tools-to-catalyst-cloud-platform</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>commercial investigation</t>
+          <t>commercial research</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>AI Coding</t>
+          <t>AI Software</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>AI coding costs could exceed developer salaries by 2028</t>
+          <t>Zoho adds AI tools to Catalyst cloud platform</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>48.6</v>
+        <v>49.7</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1257,17 +1307,22 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>pricing</t>
+          <t>listicle</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>["ai coding costs could exceed developer salaries by 2028 pricing", "ai coding costs could exceed developer salaries by 2028 faq", "how to use ai coding costs could exceed developer salaries by 2028", "ai coding costs could exceed developer salaries by 2028 alternatives", "ai coding costs could exceed developer salaries by 2028 comparison"]</t>
+          <t>["zoho adds ai tools to catalyst cloud platform faq", "zoho adds ai tools to catalyst cloud platform comparison", "zoho adds ai tools to catalyst cloud platform pricing", "how to use zoho adds ai tools to catalyst cloud platform", "zoho adds ai tools to catalyst cloud platform alternatives"]</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>["Detected search intent 'transactional' from the query.", "Matched intent terms: cost.", "Matched article-type terms: cost.", "Intent confidence 0.95; article-type confidence 0.95.", "Detected search intent 'transactional' from the query.", "Intent depth classified as deep based on query specificity."]</t>
+          <t>["Detected search intent 'commercial' from the query.", "Intent confidence 0.0; article-type confidence 0.0.", "Detected search intent 'informational' from the query.", "Intent depth classified as shallow based on query specificity.", "Scope classified as broad based on narrowing terms and product intent.", "Buyer journey stage is awareness and funnel stage is top."]</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>["bing_trending"]</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1360,7 +1415,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1370,27 +1425,27 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>best ai productivity software</t>
+          <t>open-code-review Review 2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>best-ai-productivity-software</t>
+          <t>open-code-review-review-2026</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>best ai productivity software</t>
+          <t>open-code-review Review 2026</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>best ai productivity software</t>
+          <t>open-code-review Review 2026</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>best-ai-productivity-software</t>
+          <t>open-code-review-review-2026</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1400,32 +1455,176 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>open-code-review Review 2026</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>commercial research</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>["open-code-review review 2026 alternatives", "how to use open-code-review review 2026", "open-code-review review 2026 faq", "open-code-review review 2026 comparison", "open-code-review review 2026 pricing"]</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>["Monday editorial expansion for open-code-review Review 2026.", "Detected search intent 'commercial' from the query.", "Matched intent terms: review.", "Matched article-type terms: review."]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Adobe Acquires Indian AI Startup Rilo for Marketing Automation</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>adobe-acquires-indian-ai-startup-rilo-for-marketing-automation</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Adobe Acquires Indian AI Startup Rilo for Marketing Automation</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Adobe Acquires Indian AI Startup Rilo for Marketing Automation</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>adobe-acquires-indian-ai-startup-rilo-for-marketing-automation</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>pillar</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>news/update</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Adobe Acquires Indian AI Startup Rilo for Marketing Automation</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>mixed informational and commercial</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>["adobe acquires indian ai startup rilo for marketing automation alternatives", "adobe acquires indian ai startup rilo for marketing automation faq", "adobe acquires indian ai startup rilo for marketing automation pricing", "adobe acquires indian ai startup rilo for marketing automation comparison", "how to use adobe acquires indian ai startup rilo for marketing automation"]</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>["Monday editorial expansion for Adobe Acquires Indian AI Startup Rilo for Marketing Automation.", "Detected search intent 'commercial' from the query.", "Intent confidence 0.0; article-type confidence 0.0.", "Detected search intent 'informational' from the query."]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>We Tested the 10 Best AI Productivity Tools in 2026</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>we-tested-the-10-best-ai-productivity-tools-in-2026</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>We Tested the 10 Best AI Productivity Tools in 2026</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>We Tested the 10 Best AI Productivity Tools in 2026</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>we-tested-the-10-best-ai-productivity-tools-in-2026</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>pillar</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
           <t>listicle</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>best ai productivity software</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>We Tested the 10 Best AI Productivity Tools in 2026</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>commercial research</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>["how to use best ai productivity software", "best ai productivity software comparison", "best ai productivity software faq", "best ai productivity software alternatives", "best ai productivity software pricing"]</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>["Monday editorial expansion for best ai productivity software.", "Detected search intent 'commercial' from the query.", "Matched intent terms: best.", "Matched article-type terms: best."]</t>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>["we tested the 10 best ai productivity tools in 2026 comparison", "we tested the 10 best ai productivity tools in 2026 pricing", "we tested the 10 best ai productivity tools in 2026 alternatives", "how to use we tested the 10 best ai productivity tools in 2026", "we tested the 10 best ai productivity tools in 2026 faq"]</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>["Monday editorial expansion for We Tested the 10 Best AI Productivity Tools in 2026.", "Detected search intent 'commercial' from the query.", "Matched intent terms: best.", "Matched article-type terms: best."]</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2491,6 +2690,90 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>open-code-review-review-2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>open-code-review Review 2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="D4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-09-14T12:46:04.033010+00:00</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>adobe-acquires-indian-ai-startup-rilo-for-marketing-automation</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Adobe Acquires Indian AI Startup Rilo for Marketing Automation</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="D5" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-09-14T12:46:08.171544+00:00</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>we-tested-the-10-best-ai-productivity-tools-in-2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>We Tested the 10 Best AI Productivity Tools in 2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-09-14T12:46:11.318272+00:00</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2503,14 +2786,499 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>empty</t>
-        </is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>slug</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>missing_sources</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>missing_verified_sources</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>missing_competitors</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>missing_entities</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>missing_affiliate_data</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>source_status</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>source_confidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TradingAgents Review 2026</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>tradingagents-review-2026</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; 0 usable sources below critical minimum 1; research_quality_score 45.14 below initial threshold 50.0; total_verified_source_score 0.0 below 35.0; official_docs_score 0.0 below 20.0; verified_sources 0 below 2; official_verified_sources 0 below 1; entity_coverage_score 36.0 below initial threshold 40.0; competitor_coverage_score 10.0 below initial threshold 30.0; freshness_score 0.0 below initial threshold 40.0</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026-09-14T12:44:35.964612+00:00</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>45.14</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Import AI 465: Open vs closed gaps; Kimi K3; Demis' big policy plan</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>import-ai-465-open-vs-closed-gaps-kimi-k3-demis-big-policy-plan</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; 0 usable sources below critical minimum 1; research_quality_score 47.43 below initial threshold 50.0; total_verified_source_score 0.0 below 35.0; official_docs_score 0.0 below 20.0; verified_sources 0 below 2; official_verified_sources 0 below 1; competitor_coverage_score 10.0 below initial threshold 30.0; freshness_score 0.0 below initial threshold 40.0</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-09-14T12:44:35.983080+00:00</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>47.43</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>When AI Does the Work: How SaaS Business Models Have to Change</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>when-ai-does-the-work-how-saas-business-models-have-to-change</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; 0 usable sources below critical minimum 1; research_quality_score 43.71 below initial threshold 50.0; total_verified_source_score 0.0 below 35.0; official_docs_score 0.0 below 20.0; verified_sources 0 below 2; official_verified_sources 0 below 1; entity_coverage_score 36.0 below initial threshold 40.0; competitor_coverage_score 10.0 below initial threshold 30.0; freshness_score 0.0 below initial threshold 40.0</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026-09-14T12:44:36.004175+00:00</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>43.71</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Paid: Reshaping SaaS Monetisation for Agentic AI Models</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>paid-reshaping-saas-monetisation-for-agentic-ai-models</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>13</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; 0 usable sources below critical minimum 1; research_quality_score 43.71 below initial threshold 50.0; total_verified_source_score 0.0 below 35.0; official_docs_score 0.0 below 20.0; verified_sources 0 below 2; official_verified_sources 0 below 1; entity_coverage_score 36.0 below initial threshold 40.0; competitor_coverage_score 10.0 below initial threshold 30.0; freshness_score 0.0 below initial threshold 40.0</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-09-14T12:44:36.022274+00:00</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>43.71</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5 AI Tools That Are Secretly Replacing Your Job Right Now</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>5-ai-tools-that-are-secretly-replacing-your-job-right-now</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>7</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; 0 usable sources below critical minimum 1; research_quality_score 43.71 below initial threshold 50.0; total_verified_source_score 0.0 below 35.0; official_docs_score 0.0 below 20.0; verified_sources 0 below 2; official_verified_sources 0 below 1; entity_coverage_score 36.0 below initial threshold 40.0; competitor_coverage_score 10.0 below initial threshold 30.0; freshness_score 0.0 below initial threshold 40.0</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-09-14T12:44:36.041073+00:00</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>43.71</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Organizations build software in-house using agentic coding tools instead of buying</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>organizations-build-software-in-house-using-agentic-coding-tools-instead-of-buying</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>8</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; 0 usable sources below critical minimum 1; research_quality_score 43.71 below initial threshold 50.0; total_verified_source_score 0.0 below 35.0; official_docs_score 0.0 below 20.0; verified_sources 0 below 2; official_verified_sources 0 below 1; entity_coverage_score 36.0 below initial threshold 40.0; competitor_coverage_score 10.0 below initial threshold 30.0; freshness_score 0.0 below initial threshold 40.0</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-09-14T12:44:36.076009+00:00</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>43.71</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Zoho adds AI tools to Catalyst cloud platform</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>zoho-adds-ai-tools-to-catalyst-cloud-platform</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>7</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; 0 usable sources below critical minimum 1; research_quality_score 43.71 below initial threshold 50.0; total_verified_source_score 0.0 below 35.0; official_docs_score 0.0 below 20.0; verified_sources 0 below 2; official_verified_sources 0 below 1; entity_coverage_score 36.0 below initial threshold 40.0; competitor_coverage_score 10.0 below initial threshold 30.0; freshness_score 0.0 below initial threshold 40.0</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-09-14T12:44:36.111243+00:00</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>43.71</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2600,7 +3368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2713,29 +3481,29 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>copilot-sdk-review-2026-security-and-privacy-comparison-and-alternatives</t>
+          <t>we-tested-the-10-best-ai-productivity-tools-in-2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>copilot-sdk review 2026: security and privacy comparison and alternatives</t>
+          <t>We Tested the 10 Best AI Productivity Tools in 2026</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>54.43</v>
+        <v>60.79</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
       </c>
       <c r="E2" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="F2" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -2745,34 +3513,34 @@
         <v>80</v>
       </c>
       <c r="J2" t="n">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="K2" t="n">
-        <v>54</v>
+        <v>78.5</v>
       </c>
       <c r="L2" t="n">
-        <v>20</v>
+        <v>96</v>
       </c>
       <c r="M2" t="n">
-        <v>20</v>
+        <v>95</v>
       </c>
       <c r="N2" t="n">
-        <v>10</v>
+        <v>92</v>
       </c>
       <c r="O2" t="n">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="P2" t="n">
-        <v>80</v>
+        <v>81.59</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>needs_review</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -2782,741 +3550,12 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Notion", "Gamma", "Notion AI"]</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\copilot-sdk-review-2026-security-and-privacy-comparison-and-alternatives</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>how-to-implement-copilot-sdk-review-2026-security-and-privacy</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>how to implement copilot-sdk review 2026: security and privacy</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>50.71</v>
-      </c>
-      <c r="D3" t="n">
-        <v>72</v>
-      </c>
-      <c r="E3" t="n">
-        <v>36</v>
-      </c>
-      <c r="F3" t="n">
-        <v>36</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>68</v>
-      </c>
-      <c r="I3" t="n">
-        <v>70</v>
-      </c>
-      <c r="J3" t="n">
-        <v>45</v>
-      </c>
-      <c r="K3" t="n">
-        <v>54</v>
-      </c>
-      <c r="L3" t="n">
-        <v>20</v>
-      </c>
-      <c r="M3" t="n">
-        <v>20</v>
-      </c>
-      <c r="N3" t="n">
-        <v>10</v>
-      </c>
-      <c r="O3" t="n">
-        <v>70</v>
-      </c>
-      <c r="P3" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\how-to-implement-copilot-sdk-review-2026-security-and-privacy</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>best-copilot-sdk-review-2026-workflows-and-use-cases-security</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>copilot-sdk review 2026: security and privacy</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>52.14</v>
-      </c>
-      <c r="D4" t="n">
-        <v>72</v>
-      </c>
-      <c r="E4" t="n">
-        <v>36</v>
-      </c>
-      <c r="F4" t="n">
-        <v>36</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>68</v>
-      </c>
-      <c r="I4" t="n">
-        <v>80</v>
-      </c>
-      <c r="J4" t="n">
-        <v>45</v>
-      </c>
-      <c r="K4" t="n">
-        <v>54</v>
-      </c>
-      <c r="L4" t="n">
-        <v>20</v>
-      </c>
-      <c r="M4" t="n">
-        <v>20</v>
-      </c>
-      <c r="N4" t="n">
-        <v>10</v>
-      </c>
-      <c r="O4" t="n">
-        <v>70</v>
-      </c>
-      <c r="P4" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\best-copilot-sdk-review-2026-workflows-and-use-cases-security</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>best-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-workflows-and-use-cases-pricing</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>ai in healthcare marketing: moving from automation to intelligent engagement: pricing, cost, and roi</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>60.86</v>
-      </c>
-      <c r="D5" t="n">
-        <v>72</v>
-      </c>
-      <c r="E5" t="n">
-        <v>60</v>
-      </c>
-      <c r="F5" t="n">
-        <v>60</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>68</v>
-      </c>
-      <c r="I5" t="n">
-        <v>70</v>
-      </c>
-      <c r="J5" t="n">
-        <v>61</v>
-      </c>
-      <c r="K5" t="n">
-        <v>85</v>
-      </c>
-      <c r="L5" t="n">
-        <v>20</v>
-      </c>
-      <c r="M5" t="n">
-        <v>20</v>
-      </c>
-      <c r="N5" t="n">
-        <v>10</v>
-      </c>
-      <c r="O5" t="n">
-        <v>70</v>
-      </c>
-      <c r="P5" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>ready</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited"]</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>["Make", "AdCreative AI", "Zapier"]</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\best-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-workflows-and-use-cases-pricing</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>fpt-software</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>FPT Software</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>55.14</v>
-      </c>
-      <c r="D6" t="n">
-        <v>72</v>
-      </c>
-      <c r="E6" t="n">
-        <v>36</v>
-      </c>
-      <c r="F6" t="n">
-        <v>36</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>68</v>
-      </c>
-      <c r="I6" t="n">
-        <v>70</v>
-      </c>
-      <c r="J6" t="n">
-        <v>45</v>
-      </c>
-      <c r="K6" t="n">
-        <v>85</v>
-      </c>
-      <c r="L6" t="n">
-        <v>20</v>
-      </c>
-      <c r="M6" t="n">
-        <v>20</v>
-      </c>
-      <c r="N6" t="n">
-        <v>10</v>
-      </c>
-      <c r="O6" t="n">
-        <v>70</v>
-      </c>
-      <c r="P6" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\fpt-software</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>tooljet-review-2026</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ToolJet Review 2026</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>52.14</v>
-      </c>
-      <c r="D7" t="n">
-        <v>72</v>
-      </c>
-      <c r="E7" t="n">
-        <v>36</v>
-      </c>
-      <c r="F7" t="n">
-        <v>36</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>68</v>
-      </c>
-      <c r="I7" t="n">
-        <v>80</v>
-      </c>
-      <c r="J7" t="n">
-        <v>45</v>
-      </c>
-      <c r="K7" t="n">
-        <v>54</v>
-      </c>
-      <c r="L7" t="n">
-        <v>20</v>
-      </c>
-      <c r="M7" t="n">
-        <v>20</v>
-      </c>
-      <c r="N7" t="n">
-        <v>10</v>
-      </c>
-      <c r="O7" t="n">
-        <v>70</v>
-      </c>
-      <c r="P7" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\tooljet-review-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>common-ai-accounting-automation-software-comparison-mistakes-and-troubleshooting</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>common ai accounting automation software comparison mistakes and troubleshooting</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>64.56999999999999</v>
-      </c>
-      <c r="D8" t="n">
-        <v>72</v>
-      </c>
-      <c r="E8" t="n">
-        <v>76</v>
-      </c>
-      <c r="F8" t="n">
-        <v>76</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
-        </is>
-      </c>
-      <c r="H8" t="n">
-        <v>68</v>
-      </c>
-      <c r="I8" t="n">
-        <v>80</v>
-      </c>
-      <c r="J8" t="n">
-        <v>61</v>
-      </c>
-      <c r="K8" t="n">
-        <v>85</v>
-      </c>
-      <c r="L8" t="n">
-        <v>20</v>
-      </c>
-      <c r="M8" t="n">
-        <v>20</v>
-      </c>
-      <c r="N8" t="n">
-        <v>10</v>
-      </c>
-      <c r="O8" t="n">
-        <v>70</v>
-      </c>
-      <c r="P8" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>ready</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited"]</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>["Make", "Zapier"]</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\common-ai-accounting-automation-software-comparison-mistakes-and-troubleshooting</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>ai-contract-review-tools-for-small-business</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>ai contract review tools for small business</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>47.43</v>
-      </c>
-      <c r="D9" t="n">
-        <v>72</v>
-      </c>
-      <c r="E9" t="n">
-        <v>52</v>
-      </c>
-      <c r="F9" t="n">
-        <v>52</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H9" t="n">
-        <v>68</v>
-      </c>
-      <c r="I9" t="n">
-        <v>80</v>
-      </c>
-      <c r="J9" t="n">
-        <v>45</v>
-      </c>
-      <c r="K9" t="n">
-        <v>5</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited"]</t>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\ai-contract-review-tools-for-small-business</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>ai-accounting-automation-software-comparison</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>ai accounting automation software comparison</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>59.57</v>
-      </c>
-      <c r="D10" t="n">
-        <v>72</v>
-      </c>
-      <c r="E10" t="n">
-        <v>76</v>
-      </c>
-      <c r="F10" t="n">
-        <v>76</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
-        <v>68</v>
-      </c>
-      <c r="I10" t="n">
-        <v>80</v>
-      </c>
-      <c r="J10" t="n">
-        <v>61</v>
-      </c>
-      <c r="K10" t="n">
-        <v>50</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>["official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited"]</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>["Make", "Zapier"]</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\ai-accounting-automation-software-comparison</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>is-ai-productivity-tools-pricing-worth-it-for-small-business</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>is ai productivity tools pricing worth it for small business</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>63.07</v>
-      </c>
-      <c r="D11" t="n">
-        <v>72</v>
-      </c>
-      <c r="E11" t="n">
-        <v>76</v>
-      </c>
-      <c r="F11" t="n">
-        <v>76</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>68</v>
-      </c>
-      <c r="I11" t="n">
-        <v>70</v>
-      </c>
-      <c r="J11" t="n">
-        <v>57</v>
-      </c>
-      <c r="K11" t="n">
-        <v>88.5</v>
-      </c>
-      <c r="L11" t="n">
-        <v>98</v>
-      </c>
-      <c r="M11" t="n">
-        <v>98</v>
-      </c>
-      <c r="N11" t="n">
-        <v>95</v>
-      </c>
-      <c r="O11" t="n">
-        <v>77</v>
-      </c>
-      <c r="P11" t="n">
-        <v>91.59999999999999</v>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>ready</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited"]</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>["Notion", "Gamma", "Notion AI"]</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\is-ai-productivity-tools-pricing-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\we-tested-the-10-best-ai-productivity-tools-in-2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish exact approved article how-to-implement-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10">
@@ -3368,7 +3368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3481,16 +3481,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>we-tested-the-10-best-ai-productivity-tools-in-2026</t>
+          <t>how-to-implement-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>We Tested the 10 Best AI Productivity Tools in 2026</t>
+          <t>how to implement AI In Healthcare Marketing: Moving From Automation To Intelligent Engagement</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>60.79</v>
+        <v>60.86</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
@@ -3510,52 +3510,781 @@
         <v>68</v>
       </c>
       <c r="I2" t="n">
+        <v>70</v>
+      </c>
+      <c r="J2" t="n">
+        <v>61</v>
+      </c>
+      <c r="K2" t="n">
+        <v>85</v>
+      </c>
+      <c r="L2" t="n">
+        <v>20</v>
+      </c>
+      <c r="M2" t="n">
+        <v>20</v>
+      </c>
+      <c r="N2" t="n">
+        <v>10</v>
+      </c>
+      <c r="O2" t="n">
+        <v>70</v>
+      </c>
+      <c r="P2" t="n">
         <v>80</v>
       </c>
-      <c r="J2" t="n">
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>["competitor coverage is limited"]</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>["Make", "AdCreative AI", "Zapier"]</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\how-to-implement-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>zoho-adds-ai-tools-to-catalyst-cloud-platform</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Zoho adds AI tools to Catalyst cloud platform</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>43.71</v>
+      </c>
+      <c r="D3" t="n">
+        <v>72</v>
+      </c>
+      <c r="E3" t="n">
+        <v>36</v>
+      </c>
+      <c r="F3" t="n">
+        <v>36</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>68</v>
+      </c>
+      <c r="I3" t="n">
+        <v>70</v>
+      </c>
+      <c r="J3" t="n">
+        <v>45</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\zoho-adds-ai-tools-to-catalyst-cloud-platform</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>we-tested-the-10-best-ai-productivity-tools-in-2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>We Tested the 10 Best AI Productivity Tools in 2026</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>60.79</v>
+      </c>
+      <c r="D4" t="n">
+        <v>72</v>
+      </c>
+      <c r="E4" t="n">
+        <v>60</v>
+      </c>
+      <c r="F4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>68</v>
+      </c>
+      <c r="I4" t="n">
+        <v>80</v>
+      </c>
+      <c r="J4" t="n">
         <v>57</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K4" t="n">
         <v>78.5</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L4" t="n">
         <v>96</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M4" t="n">
         <v>95</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N4" t="n">
         <v>92</v>
       </c>
-      <c r="O2" t="n">
+      <c r="O4" t="n">
         <v>57</v>
       </c>
-      <c r="P2" t="n">
+      <c r="P4" t="n">
         <v>81.59</v>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>needs_review</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>ready</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>["competitor coverage is limited"]</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>["Notion", "Gamma", "Notion AI"]</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>D:\AFFILATE BOT\data\research\we-tested-the-10-best-ai-productivity-tools-in-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>organizations-build-software-in-house-using-agentic-coding-tools-instead-of-buying</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Organizations build software in-house using agentic coding tools instead of buying</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>43.71</v>
+      </c>
+      <c r="D5" t="n">
+        <v>72</v>
+      </c>
+      <c r="E5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F5" t="n">
+        <v>36</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>68</v>
+      </c>
+      <c r="I5" t="n">
+        <v>70</v>
+      </c>
+      <c r="J5" t="n">
+        <v>45</v>
+      </c>
+      <c r="K5" t="n">
+        <v>5</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\organizations-build-software-in-house-using-agentic-coding-tools-instead-of-buying</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>adobe-acquires-indian-ai-startup-rilo-for-marketing-automation</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Adobe Acquires Indian AI Startup Rilo for Marketing Automation</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>55.86</v>
+      </c>
+      <c r="D6" t="n">
+        <v>72</v>
+      </c>
+      <c r="E6" t="n">
+        <v>60</v>
+      </c>
+      <c r="F6" t="n">
+        <v>60</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>68</v>
+      </c>
+      <c r="I6" t="n">
+        <v>70</v>
+      </c>
+      <c r="J6" t="n">
+        <v>61</v>
+      </c>
+      <c r="K6" t="n">
+        <v>50</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>["official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited"]</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>["Make", "AdCreative AI", "Zapier"]</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\adobe-acquires-indian-ai-startup-rilo-for-marketing-automation</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>5-ai-tools-that-are-secretly-replacing-your-job-right-now</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>5 AI Tools That Are Secretly Replacing Your Job Right Now</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>43.71</v>
+      </c>
+      <c r="D7" t="n">
+        <v>72</v>
+      </c>
+      <c r="E7" t="n">
+        <v>36</v>
+      </c>
+      <c r="F7" t="n">
+        <v>36</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>68</v>
+      </c>
+      <c r="I7" t="n">
+        <v>70</v>
+      </c>
+      <c r="J7" t="n">
+        <v>45</v>
+      </c>
+      <c r="K7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\5-ai-tools-that-are-secretly-replacing-your-job-right-now</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>paid-reshaping-saas-monetisation-for-agentic-ai-models</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Paid: Reshaping SaaS Monetisation for Agentic AI Models</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>43.71</v>
+      </c>
+      <c r="D8" t="n">
+        <v>72</v>
+      </c>
+      <c r="E8" t="n">
+        <v>36</v>
+      </c>
+      <c r="F8" t="n">
+        <v>36</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>68</v>
+      </c>
+      <c r="I8" t="n">
+        <v>70</v>
+      </c>
+      <c r="J8" t="n">
+        <v>45</v>
+      </c>
+      <c r="K8" t="n">
+        <v>5</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\paid-reshaping-saas-monetisation-for-agentic-ai-models</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>when-ai-does-the-work-how-saas-business-models-have-to-change</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>When AI Does the Work: How SaaS Business Models Have to Change</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>43.71</v>
+      </c>
+      <c r="D9" t="n">
+        <v>72</v>
+      </c>
+      <c r="E9" t="n">
+        <v>36</v>
+      </c>
+      <c r="F9" t="n">
+        <v>36</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>68</v>
+      </c>
+      <c r="I9" t="n">
+        <v>70</v>
+      </c>
+      <c r="J9" t="n">
+        <v>45</v>
+      </c>
+      <c r="K9" t="n">
+        <v>5</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\when-ai-does-the-work-how-saas-business-models-have-to-change</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>import-ai-465-open-vs-closed-gaps-kimi-k3-demis-big-policy-plan</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Import AI 465: Open vs closed gaps; Kimi K3; Demis' big policy plan</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>47.43</v>
+      </c>
+      <c r="D10" t="n">
+        <v>72</v>
+      </c>
+      <c r="E10" t="n">
+        <v>52</v>
+      </c>
+      <c r="F10" t="n">
+        <v>52</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>68</v>
+      </c>
+      <c r="I10" t="n">
+        <v>80</v>
+      </c>
+      <c r="J10" t="n">
+        <v>45</v>
+      </c>
+      <c r="K10" t="n">
+        <v>5</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited"]</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\import-ai-465-open-vs-closed-gaps-kimi-k3-demis-big-policy-plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>tradingagents-review-2026</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TradingAgents Review 2026</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>45.14</v>
+      </c>
+      <c r="D11" t="n">
+        <v>72</v>
+      </c>
+      <c r="E11" t="n">
+        <v>36</v>
+      </c>
+      <c r="F11" t="n">
+        <v>36</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>68</v>
+      </c>
+      <c r="I11" t="n">
+        <v>80</v>
+      </c>
+      <c r="J11" t="n">
+        <v>45</v>
+      </c>
+      <c r="K11" t="n">
+        <v>5</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\tradingagents-review-2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish exact approved article univer-review-2026
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10">
@@ -3481,42 +3481,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>how-to-implement-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement</t>
+          <t>up-review-2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>how to implement AI In Healthcare Marketing: Moving From Automation To Intelligent Engagement</t>
+          <t>up Review 2026</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>60.86</v>
+        <v>52.14</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
       </c>
       <c r="E2" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="F2" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H2" t="n">
         <v>68</v>
       </c>
       <c r="I2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J2" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="K2" t="n">
-        <v>85</v>
+        <v>54</v>
       </c>
       <c r="L2" t="n">
         <v>20</v>
@@ -3540,38 +3540,38 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>needs enrichment</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>["Make", "AdCreative AI", "Zapier"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\how-to-implement-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement</t>
+          <t>D:\AFFILATE BOT\data\research\up-review-2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>zoho-adds-ai-tools-to-catalyst-cloud-platform</t>
+          <t>univer-review-2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Zoho adds AI tools to Catalyst cloud platform</t>
+          <t>univer Review 2026</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>43.71</v>
+        <v>52.14</v>
       </c>
       <c r="D3" t="n">
         <v>72</v>
@@ -3591,32 +3591,32 @@
         <v>68</v>
       </c>
       <c r="I3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J3" t="n">
         <v>45</v>
       </c>
       <c r="K3" t="n">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O3" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -3636,23 +3636,23 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\zoho-adds-ai-tools-to-catalyst-cloud-platform</t>
+          <t>D:\AFFILATE BOT\data\research\univer-review-2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>we-tested-the-10-best-ai-productivity-tools-in-2026</t>
+          <t>implementing-intelligent-ai-healthcare-marketing-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>We Tested the 10 Best AI Productivity Tools in 2026</t>
+          <t>Implementing Intelligent AI Healthcare Marketing pricing cost and ROI</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>60.79</v>
+        <v>60.86</v>
       </c>
       <c r="D4" t="n">
         <v>72</v>
@@ -3672,32 +3672,32 @@
         <v>68</v>
       </c>
       <c r="I4" t="n">
+        <v>70</v>
+      </c>
+      <c r="J4" t="n">
+        <v>61</v>
+      </c>
+      <c r="K4" t="n">
+        <v>85</v>
+      </c>
+      <c r="L4" t="n">
+        <v>20</v>
+      </c>
+      <c r="M4" t="n">
+        <v>20</v>
+      </c>
+      <c r="N4" t="n">
+        <v>10</v>
+      </c>
+      <c r="O4" t="n">
+        <v>70</v>
+      </c>
+      <c r="P4" t="n">
         <v>80</v>
       </c>
-      <c r="J4" t="n">
-        <v>57</v>
-      </c>
-      <c r="K4" t="n">
-        <v>78.5</v>
-      </c>
-      <c r="L4" t="n">
-        <v>96</v>
-      </c>
-      <c r="M4" t="n">
-        <v>95</v>
-      </c>
-      <c r="N4" t="n">
-        <v>92</v>
-      </c>
-      <c r="O4" t="n">
-        <v>57</v>
-      </c>
-      <c r="P4" t="n">
-        <v>81.59</v>
-      </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -3712,41 +3712,41 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>["Notion", "Gamma", "Notion AI"]</t>
+          <t>["AdCreative AI"]</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\we-tested-the-10-best-ai-productivity-tools-in-2026</t>
+          <t>D:\AFFILATE BOT\data\research\implementing-intelligent-ai-healthcare-marketing-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>organizations-build-software-in-house-using-agentic-coding-tools-instead-of-buying</t>
+          <t>how-to-implement-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Organizations build software in-house using agentic coding tools instead of buying</t>
+          <t>how to implement AI In Healthcare Marketing: Moving From Automation To Intelligent Engagement</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>43.71</v>
+        <v>60.86</v>
       </c>
       <c r="D5" t="n">
         <v>72</v>
       </c>
       <c r="E5" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="F5" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -3756,78 +3756,78 @@
         <v>70</v>
       </c>
       <c r="J5" t="n">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="K5" t="n">
-        <v>5</v>
+        <v>85</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Make", "AdCreative AI", "Zapier"]</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\organizations-build-software-in-house-using-agentic-coding-tools-instead-of-buying</t>
+          <t>D:\AFFILATE BOT\data\research\how-to-implement-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>adobe-acquires-indian-ai-startup-rilo-for-marketing-automation</t>
+          <t>zoho-adds-ai-tools-to-catalyst-cloud-platform</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Adobe Acquires Indian AI Startup Rilo for Marketing Automation</t>
+          <t>Zoho adds AI tools to Catalyst cloud platform</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>55.86</v>
+        <v>43.71</v>
       </c>
       <c r="D6" t="n">
         <v>72</v>
       </c>
       <c r="E6" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="F6" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -3837,10 +3837,10 @@
         <v>70</v>
       </c>
       <c r="J6" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="K6" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
@@ -3869,110 +3869,110 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>["official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited"]</t>
+          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>["Make", "AdCreative AI", "Zapier"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\adobe-acquires-indian-ai-startup-rilo-for-marketing-automation</t>
+          <t>D:\AFFILATE BOT\data\research\zoho-adds-ai-tools-to-catalyst-cloud-platform</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>5-ai-tools-that-are-secretly-replacing-your-job-right-now</t>
+          <t>we-tested-the-10-best-ai-productivity-tools-in-2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>5 AI Tools That Are Secretly Replacing Your Job Right Now</t>
+          <t>We Tested the 10 Best AI Productivity Tools in 2026</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>43.71</v>
+        <v>60.79</v>
       </c>
       <c r="D7" t="n">
         <v>72</v>
       </c>
       <c r="E7" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="F7" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
         </is>
       </c>
       <c r="H7" t="n">
         <v>68</v>
       </c>
       <c r="I7" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J7" t="n">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="K7" t="n">
-        <v>5</v>
+        <v>78.5</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>92</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>81.59</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>needs_review</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Notion", "Gamma", "Notion AI"]</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\5-ai-tools-that-are-secretly-replacing-your-job-right-now</t>
+          <t>D:\AFFILATE BOT\data\research\we-tested-the-10-best-ai-productivity-tools-in-2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>paid-reshaping-saas-monetisation-for-agentic-ai-models</t>
+          <t>organizations-build-software-in-house-using-agentic-coding-tools-instead-of-buying</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Paid: Reshaping SaaS Monetisation for Agentic AI Models</t>
+          <t>Organizations build software in-house using agentic coding tools instead of buying</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -4041,36 +4041,36 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\paid-reshaping-saas-monetisation-for-agentic-ai-models</t>
+          <t>D:\AFFILATE BOT\data\research\organizations-build-software-in-house-using-agentic-coding-tools-instead-of-buying</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>when-ai-does-the-work-how-saas-business-models-have-to-change</t>
+          <t>adobe-acquires-indian-ai-startup-rilo-for-marketing-automation</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>When AI Does the Work: How SaaS Business Models Have to Change</t>
+          <t>Adobe Acquires Indian AI Startup Rilo for Marketing Automation</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>43.71</v>
+        <v>55.86</v>
       </c>
       <c r="D9" t="n">
         <v>72</v>
       </c>
       <c r="E9" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="F9" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -4080,10 +4080,10 @@
         <v>70</v>
       </c>
       <c r="J9" t="n">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="K9" t="n">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
@@ -4112,53 +4112,53 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Make", "AdCreative AI", "Zapier"]</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\when-ai-does-the-work-how-saas-business-models-have-to-change</t>
+          <t>D:\AFFILATE BOT\data\research\adobe-acquires-indian-ai-startup-rilo-for-marketing-automation</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>import-ai-465-open-vs-closed-gaps-kimi-k3-demis-big-policy-plan</t>
+          <t>5-ai-tools-that-are-secretly-replacing-your-job-right-now</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Import AI 465: Open vs closed gaps; Kimi K3; Demis' big policy plan</t>
+          <t>5 AI Tools That Are Secretly Replacing Your Job Right Now</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>47.43</v>
+        <v>43.71</v>
       </c>
       <c r="D10" t="n">
         <v>72</v>
       </c>
       <c r="E10" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F10" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H10" t="n">
         <v>68</v>
       </c>
       <c r="I10" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J10" t="n">
         <v>45</v>
@@ -4193,7 +4193,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited"]</t>
+          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -4203,23 +4203,23 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\import-ai-465-open-vs-closed-gaps-kimi-k3-demis-big-policy-plan</t>
+          <t>D:\AFFILATE BOT\data\research\5-ai-tools-that-are-secretly-replacing-your-job-right-now</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>tradingagents-review-2026</t>
+          <t>paid-reshaping-saas-monetisation-for-agentic-ai-models</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>TradingAgents Review 2026</t>
+          <t>Paid: Reshaping SaaS Monetisation for Agentic AI Models</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>45.14</v>
+        <v>43.71</v>
       </c>
       <c r="D11" t="n">
         <v>72</v>
@@ -4239,7 +4239,7 @@
         <v>68</v>
       </c>
       <c r="I11" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J11" t="n">
         <v>45</v>
@@ -4284,7 +4284,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\tradingagents-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\paid-reshaping-saas-monetisation-for-agentic-ai-models</t>
         </is>
       </c>
     </row>

</xml_diff>